<commit_message>
Story 24.1 review: guard, grounding and parser tests; panel wording
The worker proof now records a fact from a completed 22.4 job, a quote not
at its location, a partial quote and a EUR amount labelled USD, and checks
every insert guard and immutability rule by its own message, including the
fixture reset, the migration owner and the 1,024-fact bound. The API test
withholds a fact value from a viewer who cannot open its original. The web
parser refuses unknown keys and each structural defect alone, keeps Rust's
White_Space blank rule, and the panel says the platform evaluates a rule
Zobba proposed. Published migrations and catalogues v1-v17 are pinned by
digest. The AP invoices fixture gains one row per matrix invoice.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014HARNkCaZGyxKh3tp4iZEj
</commit_message>
<xml_diff>
--- a/zobba/fixtures/documents/AP invoices.xlsx
+++ b/zobba/fixtures/documents/AP invoices.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -586,6 +586,141 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>INV-0050</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="n">
+        <v>1250</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>J. Smith</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>09/03/2026</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>INV-0051</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>1250</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>INV-0052</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>1250</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>11/03/2026</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>INV-0053</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="n">
+        <v>1250</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>J. Smith</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>12/03/2026</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>INV-0057</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>A. Jones</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>13/03/2026</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>